<commit_message>
Update simulation and configuration data
</commit_message>
<xml_diff>
--- a/Assets/Excel/excel.xlsx
+++ b/Assets/Excel/excel.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ciga\2026CIGA\Assets\Excel\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19DD83ED-CC06-456E-8736-8697F389176C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowHeight="17775" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="item" sheetId="1" r:id="rId1"/>
@@ -30,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="130">
   <si>
     <t>道具ID</t>
   </si>
@@ -329,107 +335,107 @@
     <t>血量系数。物品健康值转换为连接最大血量的倍率。</t>
   </si>
   <si>
+    <t>海底 Unity 物理材质弹性系数。</t>
+  </si>
+  <si>
+    <t>是否显示连接血量调试信息。1 显示，0 隐藏。</t>
+  </si>
+  <si>
+    <t>物品质量系数。物品重量转换为 Unity Rigidbody2D.mass 的全局倍率。</t>
+  </si>
+  <si>
+    <t>入水初速度</t>
+  </si>
+  <si>
+    <t>关卡ID</t>
+  </si>
+  <si>
+    <t>船重量（展示用）</t>
+  </si>
+  <si>
+    <t>初始距离</t>
+  </si>
+  <si>
+    <t>最大速度</t>
+  </si>
+  <si>
+    <t>关卡基础拉力</t>
+  </si>
+  <si>
+    <t>向右横力</t>
+  </si>
+  <si>
+    <t>随机道具最低数量</t>
+  </si>
+  <si>
+    <t>最低道具总重量</t>
+  </si>
+  <si>
+    <t>推荐重量（千克）</t>
+  </si>
+  <si>
+    <t>道具重量系数</t>
+  </si>
+  <si>
+    <t>风暴级别</t>
+  </si>
+  <si>
+    <t>拼凑时间（秒）</t>
+  </si>
+  <si>
+    <t>水面张力</t>
+  </si>
+  <si>
+    <t>低级</t>
+  </si>
+  <si>
+    <t>低中</t>
+  </si>
+  <si>
+    <t>中</t>
+  </si>
+  <si>
+    <t>中高</t>
+  </si>
+  <si>
+    <t>高</t>
+  </si>
+  <si>
+    <t>坚持时间(秒）</t>
+  </si>
+  <si>
+    <t>掉落速度（m/s)</t>
+  </si>
+  <si>
+    <t>受力系数</t>
+  </si>
+  <si>
+    <t>阈值系数</t>
+  </si>
+  <si>
+    <t>伤害系数</t>
+  </si>
+  <si>
+    <t>血量系数</t>
+  </si>
+  <si>
+    <t>海底 Unity 物理材质摩擦系数。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>摩擦系数</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>防御转关节频率系数。防御越高，Unity FixedJoint2D 越硬。</t>
-  </si>
-  <si>
-    <t>海底 Unity 物理材质摩擦系数。</t>
-  </si>
-  <si>
-    <t>海底 Unity 物理材质弹性系数。</t>
-  </si>
-  <si>
-    <t>是否显示连接血量调试信息。1 显示，0 隐藏。</t>
-  </si>
-  <si>
-    <t>物品质量系数。物品重量转换为 Unity Rigidbody2D.mass 的全局倍率。</t>
-  </si>
-  <si>
-    <t>入水初速度</t>
-  </si>
-  <si>
-    <t>关卡ID</t>
-  </si>
-  <si>
-    <t>船重量（展示用）</t>
-  </si>
-  <si>
-    <t>初始距离</t>
-  </si>
-  <si>
-    <t>最大速度</t>
-  </si>
-  <si>
-    <t>关卡基础拉力</t>
-  </si>
-  <si>
-    <t>向右横力</t>
-  </si>
-  <si>
-    <t>随机道具最低数量</t>
-  </si>
-  <si>
-    <t>最低道具总重量</t>
-  </si>
-  <si>
-    <t>推荐重量（千克）</t>
-  </si>
-  <si>
-    <t>道具重量系数</t>
-  </si>
-  <si>
-    <t>风暴级别</t>
-  </si>
-  <si>
-    <t>拼凑时间（秒）</t>
-  </si>
-  <si>
-    <t>水面张力</t>
-  </si>
-  <si>
-    <t>低级</t>
-  </si>
-  <si>
-    <t>低中</t>
-  </si>
-  <si>
-    <t>中</t>
-  </si>
-  <si>
-    <t>中高</t>
-  </si>
-  <si>
-    <t>高</t>
-  </si>
-  <si>
-    <t>坚持时间(秒）</t>
-  </si>
-  <si>
-    <t>掉落速度（m/s)</t>
-  </si>
-  <si>
-    <t>受力系数</t>
-  </si>
-  <si>
-    <t>阈值系数</t>
-  </si>
-  <si>
-    <t>伤害系数</t>
-  </si>
-  <si>
-    <t>血量系数</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="21">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -441,155 +447,27 @@
       <b/>
       <sz val="11"/>
       <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <sz val="9"/>
       <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -602,194 +480,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -797,256 +489,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+  <cellXfs count="7">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
@@ -1056,68 +506,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
-    <cellStyle name="货币" xfId="2" builtinId="4"/>
-    <cellStyle name="百分比" xfId="3" builtinId="5"/>
-    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
-    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
-    <cellStyle name="超链接" xfId="6" builtinId="8"/>
-    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
-    <cellStyle name="注释" xfId="8" builtinId="10"/>
-    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
-    <cellStyle name="标题" xfId="10" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
-    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="输入" xfId="16" builtinId="20"/>
-    <cellStyle name="输出" xfId="17" builtinId="21"/>
-    <cellStyle name="计算" xfId="18" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
-    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
-    <cellStyle name="汇总" xfId="21" builtinId="25"/>
-    <cellStyle name="好" xfId="22" builtinId="26"/>
-    <cellStyle name="差" xfId="23" builtinId="27"/>
-    <cellStyle name="适中" xfId="24" builtinId="28"/>
-    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
-    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
-    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
-    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
-    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1367,20 +776,20 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:K39"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L39"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="2" max="2" width="18.3583333333333" customWidth="1"/>
-    <col min="9" max="9" width="15.625" customWidth="1"/>
+    <col min="2" max="2" width="18.375" customWidth="1"/>
+    <col min="10" max="10" width="15.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1402,24 +811,27 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" t="s">
         <v>11</v>
       </c>
       <c r="C2" t="s">
@@ -1438,19 +850,22 @@
         <v>10</v>
       </c>
       <c r="H2">
+        <v>0.3</v>
+      </c>
+      <c r="I2">
         <v>2</v>
       </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
       <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
         <v>331</v>
       </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+      <c r="L2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1473,23 +888,26 @@
         <v>12</v>
       </c>
       <c r="H3">
+        <v>0.15</v>
+      </c>
+      <c r="I3">
         <v>3</v>
       </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
       <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
         <v>285</v>
       </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+      <c r="L3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" t="s">
         <v>17</v>
       </c>
       <c r="C4" t="s">
@@ -1499,7 +917,7 @@
         <v>19</v>
       </c>
       <c r="E4">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="F4">
         <v>416</v>
@@ -1508,19 +926,22 @@
         <v>60</v>
       </c>
       <c r="H4">
+        <v>0.15</v>
+      </c>
+      <c r="I4">
         <v>6</v>
       </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
       <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
         <v>176</v>
       </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+      <c r="L4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1543,23 +964,26 @@
         <v>12</v>
       </c>
       <c r="H5">
+        <v>0.2</v>
+      </c>
+      <c r="I5">
         <v>2</v>
       </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
       <c r="J5">
-        <v>285</v>
+        <v>1</v>
       </c>
       <c r="K5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+        <v>150</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" t="s">
         <v>23</v>
       </c>
       <c r="C6" t="s">
@@ -1578,23 +1002,26 @@
         <v>24</v>
       </c>
       <c r="H6">
+        <v>0.2</v>
+      </c>
+      <c r="I6">
         <v>4</v>
       </c>
-      <c r="I6">
-        <v>1</v>
-      </c>
       <c r="J6">
-        <v>256</v>
+        <v>1</v>
       </c>
       <c r="K6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
+        <v>150</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" t="s">
         <v>25</v>
       </c>
       <c r="C7" t="s">
@@ -1613,23 +1040,26 @@
         <v>12</v>
       </c>
       <c r="H7">
+        <v>0.2</v>
+      </c>
+      <c r="I7">
         <v>2</v>
       </c>
-      <c r="I7">
-        <v>1</v>
-      </c>
       <c r="J7">
-        <v>285</v>
+        <v>1</v>
       </c>
       <c r="K7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11">
+        <v>150</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" t="s">
         <v>27</v>
       </c>
       <c r="C8" t="s">
@@ -1648,23 +1078,26 @@
         <v>24</v>
       </c>
       <c r="H8">
+        <v>0.2</v>
+      </c>
+      <c r="I8">
         <v>4</v>
       </c>
-      <c r="I8">
-        <v>1</v>
-      </c>
       <c r="J8">
-        <v>256</v>
+        <v>1</v>
       </c>
       <c r="K8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" ht="13" customHeight="1" spans="1:11">
+        <v>150</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="12.95" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>29</v>
       </c>
       <c r="C9" t="s">
@@ -1683,19 +1116,22 @@
         <v>6</v>
       </c>
       <c r="H9">
+        <v>0.3</v>
+      </c>
+      <c r="I9">
         <v>3</v>
       </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
       <c r="J9">
         <v>0</v>
       </c>
       <c r="K9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1718,23 +1154,26 @@
         <v>8</v>
       </c>
       <c r="H10">
+        <v>0.15</v>
+      </c>
+      <c r="I10">
         <v>2</v>
       </c>
-      <c r="I10">
-        <v>1</v>
-      </c>
       <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10">
         <v>331</v>
       </c>
-      <c r="K10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11">
+      <c r="L10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>33</v>
       </c>
       <c r="C11" t="s">
@@ -1753,23 +1192,26 @@
         <v>12</v>
       </c>
       <c r="H11">
+        <v>0.2</v>
+      </c>
+      <c r="I11">
         <v>2</v>
       </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
       <c r="J11">
         <v>0</v>
       </c>
       <c r="K11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>34</v>
       </c>
       <c r="C12" t="s">
@@ -1788,23 +1230,26 @@
         <v>4</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>0.15</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12">
         <v>0</v>
       </c>
       <c r="K12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C13" t="s">
@@ -1823,19 +1268,22 @@
         <v>12</v>
       </c>
       <c r="H13">
+        <v>0.25</v>
+      </c>
+      <c r="I13">
         <v>3</v>
       </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
       <c r="J13">
         <v>0</v>
       </c>
       <c r="K13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1858,19 +1306,22 @@
         <v>18</v>
       </c>
       <c r="H14">
+        <v>0.15</v>
+      </c>
+      <c r="I14">
         <v>3</v>
       </c>
-      <c r="I14">
-        <v>1</v>
-      </c>
       <c r="J14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1893,19 +1344,22 @@
         <v>18</v>
       </c>
       <c r="H15">
+        <v>0.15</v>
+      </c>
+      <c r="I15">
         <v>3</v>
       </c>
-      <c r="I15">
-        <v>1</v>
-      </c>
       <c r="J15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1928,19 +1382,22 @@
         <v>18</v>
       </c>
       <c r="H16">
+        <v>0.15</v>
+      </c>
+      <c r="I16">
         <v>3</v>
       </c>
-      <c r="I16">
-        <v>1</v>
-      </c>
       <c r="J16">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1963,19 +1420,22 @@
         <v>18</v>
       </c>
       <c r="H17">
+        <v>0.15</v>
+      </c>
+      <c r="I17">
         <v>3</v>
       </c>
-      <c r="I17">
-        <v>1</v>
-      </c>
       <c r="J17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1998,23 +1458,26 @@
         <v>12</v>
       </c>
       <c r="H18">
+        <v>0.2</v>
+      </c>
+      <c r="I18">
         <v>2</v>
       </c>
-      <c r="I18">
-        <v>0</v>
-      </c>
       <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
         <v>285</v>
       </c>
-      <c r="K18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11">
+      <c r="L18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A19">
         <v>18</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="4" t="s">
         <v>50</v>
       </c>
       <c r="C19" t="s">
@@ -2033,23 +1496,26 @@
         <v>30</v>
       </c>
       <c r="H19">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19">
         <v>0</v>
       </c>
       <c r="K19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A20">
         <v>19</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>52</v>
       </c>
       <c r="C20" t="s">
@@ -2059,7 +1525,7 @@
         <v>53</v>
       </c>
       <c r="E20">
-        <v>0.07</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F20">
         <v>60</v>
@@ -2068,23 +1534,26 @@
         <v>8</v>
       </c>
       <c r="H20">
+        <v>0.1</v>
+      </c>
+      <c r="I20">
         <v>2</v>
       </c>
-      <c r="I20">
-        <v>0</v>
-      </c>
       <c r="J20">
         <v>0</v>
       </c>
       <c r="K20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A21">
         <v>20</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="4" t="s">
         <v>54</v>
       </c>
       <c r="C21" t="s">
@@ -2103,23 +1572,26 @@
         <v>30</v>
       </c>
       <c r="H21">
+        <v>0.2</v>
+      </c>
+      <c r="I21">
         <v>5</v>
       </c>
-      <c r="I21">
-        <v>0</v>
-      </c>
       <c r="J21">
         <v>0</v>
       </c>
       <c r="K21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A22">
         <v>21</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C22" t="s">
@@ -2129,7 +1601,7 @@
         <v>49</v>
       </c>
       <c r="E22">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="F22">
         <v>13</v>
@@ -2138,23 +1610,26 @@
         <v>6</v>
       </c>
       <c r="H22">
+        <v>0.1</v>
+      </c>
+      <c r="I22">
         <v>2</v>
       </c>
-      <c r="I22">
-        <v>0</v>
-      </c>
       <c r="J22">
         <v>0</v>
       </c>
       <c r="K22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A23">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" t="s">
         <v>57</v>
       </c>
       <c r="C23" t="s">
@@ -2173,23 +1648,26 @@
         <v>15</v>
       </c>
       <c r="H23">
+        <v>0.3</v>
+      </c>
+      <c r="I23">
         <v>3</v>
       </c>
-      <c r="I23">
-        <v>0</v>
-      </c>
       <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
         <v>285</v>
       </c>
-      <c r="K23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11">
+      <c r="L23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A24">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" t="s">
         <v>59</v>
       </c>
       <c r="C24" t="s">
@@ -2208,23 +1686,26 @@
         <v>2</v>
       </c>
       <c r="H24">
+        <v>0.4</v>
+      </c>
+      <c r="I24">
         <v>4</v>
       </c>
-      <c r="I24">
-        <v>0</v>
-      </c>
       <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
         <v>524</v>
       </c>
-      <c r="K24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11">
+      <c r="L24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A25">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" t="s">
         <v>62</v>
       </c>
       <c r="C25" t="s">
@@ -2234,7 +1715,7 @@
         <v>63</v>
       </c>
       <c r="E25">
-        <v>0.07</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F25">
         <v>60</v>
@@ -2243,23 +1724,26 @@
         <v>4</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
         <v>407</v>
       </c>
-      <c r="K25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
+      <c r="L25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A26">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" t="s">
         <v>64</v>
       </c>
       <c r="C26" t="s">
@@ -2278,23 +1762,26 @@
         <v>8</v>
       </c>
       <c r="H26">
+        <v>0.1</v>
+      </c>
+      <c r="I26">
         <v>2</v>
       </c>
-      <c r="I26">
-        <v>0</v>
-      </c>
       <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
         <v>366</v>
       </c>
-      <c r="K26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
+      <c r="L26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A27">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" t="s">
         <v>66</v>
       </c>
       <c r="C27" t="s">
@@ -2313,19 +1800,22 @@
         <v>9</v>
       </c>
       <c r="H27">
+        <v>0.1</v>
+      </c>
+      <c r="I27">
         <v>3</v>
       </c>
-      <c r="I27">
-        <v>0</v>
-      </c>
       <c r="J27">
+        <v>0</v>
+      </c>
+      <c r="K27">
         <v>285</v>
       </c>
-      <c r="K27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
+      <c r="L27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2339,7 +1829,7 @@
         <v>35</v>
       </c>
       <c r="E28">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="F28">
         <v>84</v>
@@ -2348,19 +1838,22 @@
         <v>16</v>
       </c>
       <c r="H28">
+        <v>0.25</v>
+      </c>
+      <c r="I28">
         <v>4</v>
       </c>
-      <c r="I28">
-        <v>0</v>
-      </c>
       <c r="J28">
+        <v>0</v>
+      </c>
+      <c r="K28">
         <v>397</v>
       </c>
-      <c r="K28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11">
+      <c r="L28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2383,23 +1876,26 @@
         <v>16</v>
       </c>
       <c r="H29">
+        <v>0.25</v>
+      </c>
+      <c r="I29">
         <v>4</v>
       </c>
-      <c r="I29">
-        <v>0</v>
-      </c>
       <c r="J29">
+        <v>0</v>
+      </c>
+      <c r="K29">
         <v>419</v>
       </c>
-      <c r="K29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11">
+      <c r="L29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A30">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" t="s">
         <v>70</v>
       </c>
       <c r="C30" t="s">
@@ -2409,7 +1905,7 @@
         <v>71</v>
       </c>
       <c r="E30">
-        <v>4.6</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="F30">
         <v>84</v>
@@ -2418,23 +1914,26 @@
         <v>20</v>
       </c>
       <c r="H30">
+        <v>0.25</v>
+      </c>
+      <c r="I30">
         <v>5</v>
       </c>
-      <c r="I30">
-        <v>0</v>
-      </c>
       <c r="J30">
+        <v>0</v>
+      </c>
+      <c r="K30">
         <v>400</v>
       </c>
-      <c r="K30">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11">
+      <c r="L30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A31">
         <v>30</v>
       </c>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="4" t="s">
         <v>72</v>
       </c>
       <c r="C31" t="s">
@@ -2453,23 +1952,26 @@
         <v>18</v>
       </c>
       <c r="H31">
+        <v>0.15</v>
+      </c>
+      <c r="I31">
         <v>3</v>
       </c>
-      <c r="I31">
+      <c r="J31">
         <v>2</v>
       </c>
-      <c r="J31">
-        <v>0</v>
-      </c>
       <c r="K31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A32">
         <v>31</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" t="s">
         <v>73</v>
       </c>
       <c r="C32" t="s">
@@ -2488,23 +1990,26 @@
         <v>6</v>
       </c>
       <c r="H32">
+        <v>0.1</v>
+      </c>
+      <c r="I32">
         <v>2</v>
       </c>
-      <c r="I32">
-        <v>0</v>
-      </c>
       <c r="J32">
         <v>0</v>
       </c>
       <c r="K32">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11">
+        <v>0</v>
+      </c>
+      <c r="L32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A33">
         <v>32</v>
       </c>
-      <c r="B33" s="4" t="s">
+      <c r="B33" t="s">
         <v>74</v>
       </c>
       <c r="C33" t="s">
@@ -2523,23 +2028,26 @@
         <v>12</v>
       </c>
       <c r="H33">
+        <v>0.25</v>
+      </c>
+      <c r="I33">
         <v>3</v>
       </c>
-      <c r="I33">
-        <v>0</v>
-      </c>
       <c r="J33">
+        <v>0</v>
+      </c>
+      <c r="K33">
         <v>221</v>
       </c>
-      <c r="K33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11">
+      <c r="L33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A34">
         <v>33</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" t="s">
         <v>76</v>
       </c>
       <c r="C34" t="s">
@@ -2558,23 +2066,26 @@
         <v>1</v>
       </c>
       <c r="H34">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34">
+        <v>0</v>
+      </c>
+      <c r="K34">
         <v>331</v>
       </c>
-      <c r="K34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11">
+      <c r="L34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A35">
         <v>34</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B35" t="s">
         <v>79</v>
       </c>
       <c r="C35" t="s">
@@ -2593,23 +2104,26 @@
         <v>30</v>
       </c>
       <c r="H35">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I35">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35">
+        <v>0</v>
+      </c>
+      <c r="K35">
         <v>366</v>
       </c>
-      <c r="K35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11">
+      <c r="L35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A36">
         <v>35</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" t="s">
         <v>81</v>
       </c>
       <c r="C36" t="s">
@@ -2619,7 +2133,7 @@
         <v>82</v>
       </c>
       <c r="E36">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="F36">
         <v>60</v>
@@ -2628,23 +2142,26 @@
         <v>8</v>
       </c>
       <c r="H36">
+        <v>0.1</v>
+      </c>
+      <c r="I36">
         <v>2</v>
       </c>
-      <c r="I36">
-        <v>0</v>
-      </c>
       <c r="J36">
+        <v>0</v>
+      </c>
+      <c r="K36">
         <v>309</v>
       </c>
-      <c r="K36">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11">
+      <c r="L36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A37">
         <v>36</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" t="s">
         <v>83</v>
       </c>
       <c r="C37" t="s">
@@ -2663,23 +2180,26 @@
         <v>12</v>
       </c>
       <c r="H37">
+        <v>0.25</v>
+      </c>
+      <c r="I37">
         <v>3</v>
       </c>
-      <c r="I37">
-        <v>0</v>
-      </c>
       <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
         <v>240</v>
       </c>
-      <c r="K37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11">
+      <c r="L37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A38">
         <v>37</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" t="s">
         <v>85</v>
       </c>
       <c r="C38" t="s">
@@ -2698,19 +2218,22 @@
         <v>16</v>
       </c>
       <c r="H38">
+        <v>0.25</v>
+      </c>
+      <c r="I38">
         <v>4</v>
       </c>
-      <c r="I38">
-        <v>0</v>
-      </c>
       <c r="J38">
+        <v>0</v>
+      </c>
+      <c r="K38">
         <v>256</v>
       </c>
-      <c r="K38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11">
+      <c r="L38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2733,36 +2256,38 @@
         <v>40</v>
       </c>
       <c r="H39">
+        <v>0.15</v>
+      </c>
+      <c r="I39">
         <v>4</v>
       </c>
-      <c r="I39">
-        <v>0</v>
-      </c>
       <c r="J39">
+        <v>0</v>
+      </c>
+      <c r="K39">
         <v>215</v>
       </c>
-      <c r="K39">
+      <c r="L39">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="13.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="62" style="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>89</v>
       </c>
@@ -2770,7 +2295,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>91</v>
       </c>
@@ -2778,7 +2303,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
         <v>92</v>
       </c>
@@ -2786,7 +2311,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
         <v>93</v>
       </c>
@@ -2794,31 +2319,31 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>94</v>
       </c>
       <c r="B5">
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>95</v>
       </c>
       <c r="B6">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
         <v>96</v>
       </c>
       <c r="B7">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
         <v>97</v>
       </c>
@@ -2826,120 +2351,119 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
         <v>98</v>
       </c>
       <c r="B9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A10" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B10">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A11" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="B11">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A12" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B10">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11" s="3" t="s">
+      <c r="B12">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A13" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B11">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12" s="3" t="s">
+      <c r="B13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="27" x14ac:dyDescent="0.15">
+      <c r="A14" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B12">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" s="3" t="s">
+      <c r="B14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.15">
+      <c r="A15" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" ht="27" spans="1:2">
-      <c r="A14" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="B15" s="1">
         <v>10</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="12" width="14.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" t="s">
         <v>105</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>106</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>107</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>108</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>109</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>110</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>111</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>112</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>113</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>114</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>115</v>
       </c>
-      <c r="L1" t="s">
-        <v>116</v>
-      </c>
-      <c r="M1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2954,10 +2478,10 @@
         <v>60</v>
       </c>
       <c r="E2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F2">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G2">
         <v>30</v>
@@ -2972,16 +2496,16 @@
         <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="L2">
         <v>180</v>
       </c>
       <c r="M2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2996,10 +2520,10 @@
         <v>72</v>
       </c>
       <c r="E3">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F3">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="G3">
         <v>32</v>
@@ -3008,22 +2532,22 @@
         <v>37</v>
       </c>
       <c r="I3">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="J3">
         <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="L3">
         <v>180</v>
       </c>
       <c r="M3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3038,7 +2562,7 @@
         <v>84</v>
       </c>
       <c r="E4">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F4">
         <v>1.4</v>
@@ -3050,22 +2574,22 @@
         <v>43</v>
       </c>
       <c r="I4">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="J4">
-        <v>1.05392156862745</v>
+        <v>1.0539215686274499</v>
       </c>
       <c r="K4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="L4">
         <v>180</v>
       </c>
       <c r="M4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3080,10 +2604,10 @@
         <v>96</v>
       </c>
       <c r="E5">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F5">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="G5">
         <v>36</v>
@@ -3092,22 +2616,22 @@
         <v>57</v>
       </c>
       <c r="I5">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="J5">
         <v>1.31944444444444</v>
       </c>
       <c r="K5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="L5">
         <v>180</v>
       </c>
       <c r="M5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3122,10 +2646,10 @@
         <v>108</v>
       </c>
       <c r="E6">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="G6">
         <v>38</v>
@@ -3137,19 +2661,19 @@
         <v>50</v>
       </c>
       <c r="J6">
-        <v>1.55701754385965</v>
+        <v>1.5570175438596501</v>
       </c>
       <c r="K6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L6">
         <v>180</v>
       </c>
       <c r="M6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3164,10 +2688,10 @@
         <v>120</v>
       </c>
       <c r="E7">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F7">
-        <v>2.3</v>
+        <v>2</v>
       </c>
       <c r="G7">
         <v>40</v>
@@ -3182,16 +2706,16 @@
         <v>1.75</v>
       </c>
       <c r="K7" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L7">
         <v>180</v>
       </c>
       <c r="M7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3206,10 +2730,10 @@
         <v>132</v>
       </c>
       <c r="E8">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="F8">
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="G8">
         <v>42</v>
@@ -3224,16 +2748,16 @@
         <v>1.9047619047619</v>
       </c>
       <c r="K8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L8">
         <v>180</v>
       </c>
       <c r="M8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3248,10 +2772,10 @@
         <v>144</v>
       </c>
       <c r="E9">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="F9">
-        <v>2.9</v>
+        <v>4</v>
       </c>
       <c r="G9">
         <v>44</v>
@@ -3263,19 +2787,19 @@
         <v>80</v>
       </c>
       <c r="J9">
-        <v>2.04545454545455</v>
+        <v>2.0454545454545499</v>
       </c>
       <c r="K9" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L9">
         <v>180</v>
       </c>
       <c r="M9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3290,10 +2814,10 @@
         <v>156</v>
       </c>
       <c r="E10">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="F10">
-        <v>3.2</v>
+        <v>5</v>
       </c>
       <c r="G10">
         <v>46</v>
@@ -3305,19 +2829,19 @@
         <v>90</v>
       </c>
       <c r="J10">
-        <v>2.17391304347826</v>
+        <v>2.1739130434782599</v>
       </c>
       <c r="K10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L10">
         <v>180</v>
       </c>
       <c r="M10">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.15">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3332,10 +2856,10 @@
         <v>168</v>
       </c>
       <c r="E11">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F11">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="G11">
         <v>48</v>
@@ -3347,84 +2871,83 @@
         <v>100</v>
       </c>
       <c r="J11">
-        <v>2.29166666666667</v>
+        <v>2.2916666666666701</v>
       </c>
       <c r="K11" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="L11">
         <v>180</v>
       </c>
       <c r="M11">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultColWidth="8.725" defaultRowHeight="13.5" outlineLevelRow="5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="18.725" customWidth="1"/>
+    <col min="1" max="1" width="18.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B1">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B2">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>